<commit_message>
catalogue change / order protection
</commit_message>
<xml_diff>
--- a/public/Цены.xlsx
+++ b/public/Цены.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/askerdursunov/grocery-store-webapp/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A060CB89-F5CD-3C47-BE69-4C06797F60D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE7471D9-DB38-614E-9AB6-84306EB87A62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17200" activeTab="5" xr2:uid="{7BE44800-E21B-C249-A75E-04DC14375F69}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17200" xr2:uid="{7BE44800-E21B-C249-A75E-04DC14375F69}"/>
   </bookViews>
   <sheets>
     <sheet name="Заморозка" sheetId="1" r:id="rId1"/>
@@ -43,495 +43,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="173">
   <si>
-    <t>ФЕРМАГ АДЖИКА ПО ДОМАШНЕМУ 300 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БАГЕТ 300 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БАГЕТ ЖИВАЯ РОЖЬ 300 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БАТОН МОЛОЧНЫЙ С КУНЖУТОМ (В НАРЕЗКЕ) 300 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БАТОН МОЛОЧНЫЙ С КУНЖУТОМ 300 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БАТОН НАРЕЗНОЙ (В НАРЕЗКЕ) 300 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БАТОН НАРЕЗНОЙ 300 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БАТОН ОТРУБНОЙ (В НАРЕЗКЕ) 300 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БАТОН ОТРУБНОЙ 300 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БАТОН ТУРЕЦКИЙ 250 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БАУРСАКИ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БЕЗЕ ЦВЕТНОЕ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БЕЗЕ ШОКОЛАДНОЕ С ГРЕЦКИМ ОРЕХОМ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БЛИНЫ С ТВОРОГОМ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БУЛОЧКА АЧМА С СЫРОМ 130 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БУЛОЧКА АЧМА С ШОКОЛАДОМ 130 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БУЛОЧКА АЧМА СО ШПИНАТОМ И ТВОРОГОМ 170 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БУЛОЧКА БЛИЗНЯШКА 150 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БУЛОЧКА ВАТРУШКА 100Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БУЛОЧКА ДЛЯ ГАМБУРГЕРА 3 ШТ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БУЛОЧКА ДЛЯ ХОТ-ДОГА 3 ШТ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БУЛОЧКА ПЛЕТЕНКА С МАКОМ 150 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БУЛОЧКА ПОАЧА С КАРТОШКОЙ 100 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БУЛОЧКА ПОАЧА С СЫРОМ 100 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БУЛОЧКА С ИЗЮМОМ 100Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БУЛОЧКА С КОРИЦЕЙ 100Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БУЛОЧКА СДОБНАЯ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БУЛОЧКА СЕРДЕЧКО 100Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БУЛОЧКА ЯРОСЛАВСКАЯ 100 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ БУЛОЧКИ С НАЧИНКОЙ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ВАРЕНЬЕ ВИШНЕВАЯ КОСТОЧКА 350 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ВАРЕНЬЕ ИЗ ГРУШИ 350 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ВАФЕЛЬНЫЕ ТРУБОЧКИ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ГАЛЕТА, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ГО БЕДРО В МАРИНАДЕ С ГРЕЧКОЙ 250 Г (КОМПЛЕКС №7)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ГО БЕФСТРОГАНОВ ИЗ КУРИЦЫ С ГРЕЧКОЙ 250 Г (КОМПЛЕКС №16)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ГО БЕФСТРОГАНОВ ИЗ КУРИЦЫ С РИСОМ 250 Г (КОМПЛЕКС №5)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ГО ГОЛЕНЬ ЗАПЕЧЕННАЯ С РИСОМ 250 Г (КОМПЛЕКС №6)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ГО ГУЛЯШ ИЗ ГОВЯДИНЫ С ПЮРЕ 250 Г (КОМПЛЕКС №8)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ГО КОТЛЕТА ЖАСТАР КУРИНАЯ С ПЮРЕ 250 Г (КОМПЛЕКС №9)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ГО КОТЛЕТА ИЗ ГОВЯДИНЫ С МАКАРОНАМИ 250 Г (КОМПЛЕКС №18)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ГО КОТЛЕТА ИЗ ГОВЯДИНЫ С ПЮРЕ 250 Г (КОМПЛЕКС №2)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ГО КОТЛЕТА НАУРЫЗ КУРИНАЯ С РИСОМ 250 Г (КОМПЛЕКС №1)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ГО КУРИЦА ТЕРИЯКИ С КАРТОФЕЛЬНЫМ ПЮРЕ 250 Г (КОМПЛЕКС №14)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ГО КУРИЦА ТЕРИЯКИ С РИСОМ ОТВАРНЫМ 250 Г (КОМПЛЕКС №20)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ГО МАРИНОВАННЫЕ КРЫЛЫШКИ С ГРЕЧКОЙ 250 Г (КОМПЛЕКС №17)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ГО МАРИНОВАННЫЕ КРЫЛЫШКИ С РИСОМ 250 Г (КОМПЛЕКС №15)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ГО МЯСО ПО ТАЙСКИ С РИСОМ 250 Г (КОМПЛЕКС №12)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ГО НАГГЕТСЫ С ГРЕЧКОЙ 250 Г (КОМПЛЕКС №3)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ГО НАГГЕТСЫ С ПЮРЕ 250 Г (КОМПЛЕКС №11)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ГО СУДАК С ЦВЕТНЫМ РИСОМ 250 Г (КОМПЛЕКС №19)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ГО ТЕФТЕЛИ ГОВЯЖЬИ С МАКАРОНАМИ 250 Г (КОМПЛЕКС №10)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ГО ФИЛЕ С ОВОЩАМИ С ЦВЕТНЫМ РИСОМ 250 Г (КОМПЛЕКС №13)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ДЖАДЖИК КЛАССИЧЕСКИЙ 360 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ДЖАДЖИК ПИКАНТНЫЙ 360 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ КАЛАЧ СМИТ ТУРЕЦКИЙ 1 ШТ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ КАПУСТА КВАШЕНАЯ, КГ (В)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ КАПУСТА ЦВЕТНАЯ В КЛЯРЕ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ КЕКС ТВОРОЖНЫЙ СВЕЖАЯ ЯГОДА 200 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ КОЛЬЦА ТВОРОЖНЫЕ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ КОРЗИНКА ВОСТОЧНАЯ 150 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ КОРЗИНКА ТВОРОЖНАЯ С ЯГОДОЙ 150 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ КРУАССАН С ШОКОЛАДОМ 100 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ КУТАБЫ 150 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ЛАВАШ 2 ШТ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ЛАГМАН 300 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ЛАГМАН ЖАРЕНЫЙ, КГ (В)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ЛАПША ДОМАШНЯЯ ЯИЧНАЯ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ЛЕПЕШКА РАМАЗАН 400 Г (Т)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ЛЕПЕШКА С СЫРОМ 130 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ЛЕПЕШКА ТАШКЕНТСКАЯ 400 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ МАНТЫ С КУРИЦЕЙ,ТЫКВОЙ И КАРТОШКОЙ 60 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ МАНТЫ С МЯСОМ 60 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ МИНИ ПИЦЦА 130 Г (Т)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ МИНИ ПИЦЦА НЕАПОЛИТАНСКАЯ ШТ 110 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ МОРС КЛЮКВЕННЫЙ 0,5 Л</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ МОРС МАЛИНОВЫЙ 0,5 Л</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ МОРС ОБЛЕПИХОВЫЙ 0,5 Л</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ МОРС ЯГОДНЫЙ 0,5 Л</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ОВОЩИ ГРИЛЬ, КГ (В)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ОКРОШКА С КОЛБАСОЙ 360 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ОМЛЕТ С ЗЕЛЕНЬЮ КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПАНИНИ С КУРИЦЕЙ 350 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПАСТА ЗЕЛЕНАЯ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПЕРЧИК ФАРШИРОВАННЫЙ, КГ (В)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПЕЧЕНЬ КУРИНАЯ В СМЕТАННОМ СОУСЕ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПЕЧЕНЬЕ АМЕРИКАНО, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПЕЧЕНЬЕ БИСКОНТИ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПЕЧЕНЬЕ ДОМАШНЕЕ ТВОРОЖНОЕ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПЕЧЕНЬЕ ИЗЮМИНКА, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПЕЧЕНЬЕ КУКИ С ШОКОЛАДОМ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПЕЧЕНЬЕ КУКИ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПЕЧЕНЬЕ КУРАБЬЕ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПЕЧЕНЬЕ С ПЕЧЕНЫМ ЯБЛОКОМ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПЕЧЕНЬЕ СОЛЕНОЕ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПЕЧЕНЬЕ ТАРТУС, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПИРОГ ВОСТОЧНЫЙ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПИРОГ С КУРИЦЕЙ И КАРТОШКОЙ,КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПИРОГ С МЯСОМ И КАРТОШКОЙ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПИРОГ ТВОРОЖНО-ФРУКТОВЫЙ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПИРОГ ЯБЛОЧНЫЙ С КОРИЦЕЙ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПИРОЖКИ ЖАРЕНЫЕ С КАПУСТОЙ 80 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПИРОЖКИ ЖАРЕНЫЕ С КАРТОШКОЙ 80 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПИРОЖКИ ЖАРЕНЫЕ С ЛУКОМ/ЯЙЦОМ 100 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПИРОЖКИ ПЕЧЕНЫЙ С КАПУСТОЙ 100 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПИРОЖКИ ПЕЧЕНЫЙ С КАРТОШКОЙ 100 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПИРОЖОК ПЕЧЕНЫЙ С ЯЙЦОМ ЛУКОМ 100 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПЛАЧИНДА С КУРИЦЕЙ 150Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПЛАЧИНДА С МЯСОМ 150Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПЛЕТЕНКА СО СГУЩЕНКОЙ С ГРЕЦКИМ ОРЕХОМ 150 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПЛОВ ИЗ ГОВЯДИНЫ 300 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПЛОВ ИЗ ГОВЯДИНЫ, КГ (В)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПОНЧИК БЕРЛИНСКИЙ БЕРЛИНЕР 50 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ПРОФИТРОЛИ СО ВЗБИТЫМИ СЛИВКАМИ И КРЕМОМ ЧИЗ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ РУЛЕТ МАКОВЫЙ 380 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ РУЛЕТ МЕДОВЫЙ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ РУЛЕТ ОРЕХОВЫЙ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ РУЛЕТ СО СГУЩЕНКОЙ И ГРЕЦКИМ ОРЕХОМ 380 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ РУЛЕТ ШОКОЛАДНЫЙ 500 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ САЛАТ МОРКОВЬ ПО КОРЕЙСКИ, КГ (В)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ САМСА БОЛЬШАЯ С КУРИЦЕЙ 1 ШТ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ САМСА БОЛЬШАЯ С МЯСОМ 1 ШТ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ САМСА БОЛЬШАЯ С СЫРОМ 1 ШТ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ САМСА МИКС 1 ШТ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ САМСА УЙГУРСКАЯ С МЯСОМ 1 ШТ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ САМСА ШАШЛЫК ФИЛЕ 1 ШТ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ СЛОЙКА С СЫРОМ 140 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ СЛОЙКА С ЯБЛОКОМ 140 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ СОСИСКА В ТЕСТЕ 100 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ СОСИСКА ПО-БАВАРСКИ 1 ШТ (В)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ СОЧНИК С ТВОРОГОМ 120 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ СТЕЙК СЕМГИ, КГ (В)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ СУХАРИ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ СЫРНИКИ 90 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ТЕСТО ДЛЯ БАУРСАКОВ, КГ (1)</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ТЕСТО СЛОЕНОЕ КЛАССИЧЕСКОЕ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ТОРТ МОРКОВНЫЙ КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ТОРТ МУРАВЕЙНИК, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ТОРТ ПЫЖИК МЕДОВО ШОКОЛАДНЫЙ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ТОРТ РЫЖИК МЕДОВЫЙ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ТРАЙФЛ ДЕСЕРТ 200 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ УЧПУЧМАК С МЯСОМ/КАРТОФЕЛЕМ 120 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ХВОРОСТ, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ХЛЕБ БЕЗДРОЖЖЕВОЙ РЕМЕСЛЕННЫЙ 320 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ХЛЕБ ГРЕЧИШНЫЙ 300Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ХЛЕБ ДОМАШНИЙ 460 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ХЛЕБ ЗИМНИЙ ФРУКТОВЫЙ 250 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ХЛЕБ КУКУРУЗНЫЙ (В НАРЕЗКЕ) 350 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ХЛЕБ КУКУРУЗНЫЙ 350 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ХЛЕБ НА СЫВОРОТКЕ 300 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ХЛЕБ ПОЛТАВСКИЙ 500 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ХЛЕБ ПОСОЛЬСКИЙ 400 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ХЛЕБ ПРЕЗИДЕНТСКИЙ (В НАРЕЗКЕ) 300 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ХЛЕБ ПРЕЗИДЕНТСКИЙ 300 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ХЛЕБ РЖАНОЙ 500 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ХЛЕБ РЖАНОЙ НЕМЕЦКИЙ 400 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ХЛЕБ РОМАШКА С КУНЖУТОМ 300 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ХЛЕБ ТОСТОВЫЙ 300 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ХЛЕБ ЧЕСНОЧНЫЙ 200 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ХЛЕБЦЫ ЗЛАКОВЫЕ П/П, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ЧАК-ЧАК, КГ</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ЭКЛЕРЫ С КРЕМОМ И СГУЩЕНКОЙ 120 Г</t>
-  </si>
-  <si>
-    <t>ФЕРМАГ ЭЛЕШ С КУРИЦЕЙ 150 Г</t>
-  </si>
-  <si>
     <t>САЛАТ ОЛИВЬЕ КГ</t>
   </si>
   <si>
@@ -560,6 +71,495 @@
   </si>
   <si>
     <t>САЛАТ СВЕКЛА ПОД СЫРОМ, КГ (В)</t>
+  </si>
+  <si>
+    <t>ГО БЕДРО В МАРИНАДЕ С ГРЕЧКОЙ 250 Г (КОМПЛЕКС №7)</t>
+  </si>
+  <si>
+    <t>ГО БЕФСТРОГАНОВ ИЗ КУРИЦЫ С ГРЕЧКОЙ 250 Г (КОМПЛЕКС №16)</t>
+  </si>
+  <si>
+    <t>ГО БЕФСТРОГАНОВ ИЗ КУРИЦЫ С РИСОМ 250 Г (КОМПЛЕКС №5)</t>
+  </si>
+  <si>
+    <t>ГО ГОЛЕНЬ ЗАПЕЧЕННАЯ С РИСОМ 250 Г (КОМПЛЕКС №6)</t>
+  </si>
+  <si>
+    <t>ГО ГУЛЯШ ИЗ ГОВЯДИНЫ С ПЮРЕ 250 Г (КОМПЛЕКС №8)</t>
+  </si>
+  <si>
+    <t>ГО КОТЛЕТА ЖАСТАР КУРИНАЯ С ПЮРЕ 250 Г (КОМПЛЕКС №9)</t>
+  </si>
+  <si>
+    <t>ГО КОТЛЕТА ИЗ ГОВЯДИНЫ С МАКАРОНАМИ 250 Г (КОМПЛЕКС №18)</t>
+  </si>
+  <si>
+    <t>ГО КОТЛЕТА ИЗ ГОВЯДИНЫ С ПЮРЕ 250 Г (КОМПЛЕКС №2)</t>
+  </si>
+  <si>
+    <t>ГО КОТЛЕТА НАУРЫЗ КУРИНАЯ С РИСОМ 250 Г (КОМПЛЕКС №1)</t>
+  </si>
+  <si>
+    <t>ГО КУРИЦА ТЕРИЯКИ С КАРТОФЕЛЬНЫМ ПЮРЕ 250 Г (КОМПЛЕКС №14)</t>
+  </si>
+  <si>
+    <t>ГО КУРИЦА ТЕРИЯКИ С РИСОМ ОТВАРНЫМ 250 Г (КОМПЛЕКС №20)</t>
+  </si>
+  <si>
+    <t>ГО МАРИНОВАННЫЕ КРЫЛЫШКИ С ГРЕЧКОЙ 250 Г (КОМПЛЕКС №17)</t>
+  </si>
+  <si>
+    <t>ГО МАРИНОВАННЫЕ КРЫЛЫШКИ С РИСОМ 250 Г (КОМПЛЕКС №15)</t>
+  </si>
+  <si>
+    <t>ГО МЯСО ПО ТАЙСКИ С РИСОМ 250 Г (КОМПЛЕКС №12)</t>
+  </si>
+  <si>
+    <t>ГО НАГГЕТСЫ С ГРЕЧКОЙ 250 Г (КОМПЛЕКС №3)</t>
+  </si>
+  <si>
+    <t>ГО НАГГЕТСЫ С ПЮРЕ 250 Г (КОМПЛЕКС №11)</t>
+  </si>
+  <si>
+    <t>ГО СУДАК С ЦВЕТНЫМ РИСОМ 250 Г (КОМПЛЕКС №19)</t>
+  </si>
+  <si>
+    <t>ГО ТЕФТЕЛИ ГОВЯЖЬИ С МАКАРОНАМИ 250 Г (КОМПЛЕКС №10)</t>
+  </si>
+  <si>
+    <t>ГО ФИЛЕ С ОВОЩАМИ С ЦВЕТНЫМ РИСОМ 250 Г (КОМПЛЕКС №13)</t>
+  </si>
+  <si>
+    <t>ВАРЕНЬЕ ВИШНЕВАЯ КОСТОЧКА 350 Г</t>
+  </si>
+  <si>
+    <t>ВАРЕНЬЕ ИЗ ГРУШИ 350 Г</t>
+  </si>
+  <si>
+    <t>БЕЗЕ ЦВЕТНОЕ, КГ</t>
+  </si>
+  <si>
+    <t>БЕЗЕ ШОКОЛАДНОЕ С ГРЕЦКИМ ОРЕХОМ, КГ</t>
+  </si>
+  <si>
+    <t>ВАФЕЛЬНЫЕ ТРУБОЧКИ, КГ</t>
+  </si>
+  <si>
+    <t>КЕКС ТВОРОЖНЫЙ СВЕЖАЯ ЯГОДА 200 Г</t>
+  </si>
+  <si>
+    <t>КОРЗИНКА ТВОРОЖНАЯ С ЯГОДОЙ 150 Г</t>
+  </si>
+  <si>
+    <t>КОРЗИНКА ВОСТОЧНАЯ 150 Г</t>
+  </si>
+  <si>
+    <t>КОЛЬЦА ТВОРОЖНЫЕ, КГ</t>
+  </si>
+  <si>
+    <t>ЭКЛЕРЫ С КРЕМОМ И СГУЩЕНКОЙ 120 Г</t>
+  </si>
+  <si>
+    <t>ПРОФИТРОЛИ СО ВЗБИТЫМИ СЛИВКАМИ И КРЕМОМ ЧИЗ, КГ</t>
+  </si>
+  <si>
+    <t>ПИРОГ ВОСТОЧНЫЙ, КГ</t>
+  </si>
+  <si>
+    <t>ПИРОГ ТВОРОЖНО-ФРУКТОВЫЙ, КГ</t>
+  </si>
+  <si>
+    <t>ПИРОГ ЯБЛОЧНЫЙ С КОРИЦЕЙ, КГ</t>
+  </si>
+  <si>
+    <t>РУЛЕТ ШОКОЛАДНЫЙ 500 Г</t>
+  </si>
+  <si>
+    <t>РУЛЕТ МАКОВЫЙ 380 Г</t>
+  </si>
+  <si>
+    <t>РУЛЕТ СО СГУЩЕНКОЙ И ГРЕЦКИМ ОРЕХОМ 380 Г</t>
+  </si>
+  <si>
+    <t>РУЛЕТ МЕДОВЫЙ, КГ</t>
+  </si>
+  <si>
+    <t>РУЛЕТ ОРЕХОВЫЙ, КГ</t>
+  </si>
+  <si>
+    <t>СОЧНИК С ТВОРОГОМ 120 Г</t>
+  </si>
+  <si>
+    <t>ТРАЙФЛ ДЕСЕРТ 200 Г</t>
+  </si>
+  <si>
+    <t>ХВОРОСТ, КГ</t>
+  </si>
+  <si>
+    <t>ЧАК-ЧАК, КГ</t>
+  </si>
+  <si>
+    <t>ПОНЧИК БЕРЛИНСКИЙ БЕРЛИНЕР 50 Г</t>
+  </si>
+  <si>
+    <t>ТОРТ МОРКОВНЫЙ КГ</t>
+  </si>
+  <si>
+    <t>ТОРТ МУРАВЕЙНИК, КГ</t>
+  </si>
+  <si>
+    <t>ТОРТ ПЫЖИК МЕДОВО ШОКОЛАДНЫЙ, КГ</t>
+  </si>
+  <si>
+    <t>ТОРТ РЫЖИК МЕДОВЫЙ, КГ</t>
+  </si>
+  <si>
+    <t>ПЕЧЕНЬЕ АМЕРИКАНО, КГ</t>
+  </si>
+  <si>
+    <t>ПЕЧЕНЬЕ КУКИ, КГ</t>
+  </si>
+  <si>
+    <t>ПЕЧЕНЬЕ КУКИ С ШОКОЛАДОМ, КГ</t>
+  </si>
+  <si>
+    <t>ПЕЧЕНЬЕ ИЗЮМИНКА, КГ</t>
+  </si>
+  <si>
+    <t>ПЕЧЕНЬЕ КУРАБЬЕ, КГ</t>
+  </si>
+  <si>
+    <t>ПЕЧЕНЬЕ С ПЕЧЕНЫМ ЯБЛОКОМ, КГ</t>
+  </si>
+  <si>
+    <t>ПЕЧЕНЬЕ ДОМАШНЕЕ ТВОРОЖНОЕ, КГ</t>
+  </si>
+  <si>
+    <t>ПЕЧЕНЬЕ СОЛЕНОЕ, КГ</t>
+  </si>
+  <si>
+    <t>ПЕЧЕНЬЕ ТАРТУС, КГ</t>
+  </si>
+  <si>
+    <t>ПЕЧЕНЬЕ БИСКОНТИ, КГ</t>
+  </si>
+  <si>
+    <t>САЛАТ МОРКОВЬ ПО КОРЕЙСКИ, КГ (В)</t>
+  </si>
+  <si>
+    <t>МАНТЫ С КУРИЦЕЙ,ТЫКВОЙ И КАРТОШКОЙ 60 Г</t>
+  </si>
+  <si>
+    <t>МАНТЫ С МЯСОМ 60 Г</t>
+  </si>
+  <si>
+    <t>ПАНИНИ С КУРИЦЕЙ 350 Г</t>
+  </si>
+  <si>
+    <t>МОРС КЛЮКВЕННЫЙ 0,5 Л</t>
+  </si>
+  <si>
+    <t>МОРС МАЛИНОВЫЙ 0,5 Л</t>
+  </si>
+  <si>
+    <t>МОРС ОБЛЕПИХОВЫЙ 0,5 Л</t>
+  </si>
+  <si>
+    <t>МОРС ЯГОДНЫЙ 0,5 Л</t>
+  </si>
+  <si>
+    <t>ОКРОШКА С КОЛБАСОЙ 360 Г</t>
+  </si>
+  <si>
+    <t>ДЖАДЖИК КЛАССИЧЕСКИЙ 360 Г</t>
+  </si>
+  <si>
+    <t>ДЖАДЖИК ПИКАНТНЫЙ 360 Г</t>
+  </si>
+  <si>
+    <t>АДЖИКА ПО ДОМАШНЕМУ 300 Г</t>
+  </si>
+  <si>
+    <t>ПЛОВ ИЗ ГОВЯДИНЫ 300 Г</t>
+  </si>
+  <si>
+    <t>ЛАГМАН 300 Г</t>
+  </si>
+  <si>
+    <t>ПЕРЧИК ФАРШИРОВАННЫЙ, КГ (В)</t>
+  </si>
+  <si>
+    <t>СТЕЙК СЕМГИ, КГ (В)</t>
+  </si>
+  <si>
+    <t>БЛИНЫ С ТВОРОГОМ, КГ</t>
+  </si>
+  <si>
+    <t>ПЛОВ ИЗ ГОВЯДИНЫ, КГ (В)</t>
+  </si>
+  <si>
+    <t>ЛАГМАН ЖАРЕНЫЙ, КГ (В)</t>
+  </si>
+  <si>
+    <t>БАУРСАКИ, КГ</t>
+  </si>
+  <si>
+    <t>КАПУСТА КВАШЕНАЯ, КГ (В)</t>
+  </si>
+  <si>
+    <t>ЛАПША ДОМАШНЯЯ ЯИЧНАЯ, КГ</t>
+  </si>
+  <si>
+    <t>ПАСТА ЗЕЛЕНАЯ, КГ</t>
+  </si>
+  <si>
+    <t>ПЕЧЕНЬ КУРИНАЯ В СМЕТАННОМ СОУСЕ, КГ</t>
+  </si>
+  <si>
+    <t>СЫРНИКИ 90 Г</t>
+  </si>
+  <si>
+    <t>ОМЛЕТ С ЗЕЛЕНЬЮ КГ</t>
+  </si>
+  <si>
+    <t>КАПУСТА ЦВЕТНАЯ В КЛЯРЕ, КГ</t>
+  </si>
+  <si>
+    <t>ОВОЩИ ГРИЛЬ, КГ (В)</t>
+  </si>
+  <si>
+    <t>КУТАБЫ 150 Г</t>
+  </si>
+  <si>
+    <t>ХЛЕБ ЗИМНИЙ ФРУКТОВЫЙ 250 Г</t>
+  </si>
+  <si>
+    <t>ХЛЕБ ГРЕЧИШНЫЙ 300Г</t>
+  </si>
+  <si>
+    <t>ХЛЕБ ПОЛТАВСКИЙ 500 Г</t>
+  </si>
+  <si>
+    <t>ХЛЕБ РЖАНОЙ 500 Г</t>
+  </si>
+  <si>
+    <t>ХЛЕБ ДОМАШНИЙ 460 Г</t>
+  </si>
+  <si>
+    <t>ХЛЕБ НА СЫВОРОТКЕ 300 Г</t>
+  </si>
+  <si>
+    <t>БАГЕТ 300 Г</t>
+  </si>
+  <si>
+    <t>БАГЕТ ЖИВАЯ РОЖЬ 300 Г</t>
+  </si>
+  <si>
+    <t>БАТОН МОЛОЧНЫЙ С КУНЖУТОМ 300 Г</t>
+  </si>
+  <si>
+    <t>БАТОН МОЛОЧНЫЙ С КУНЖУТОМ (В НАРЕЗКЕ) 300 Г</t>
+  </si>
+  <si>
+    <t>БАТОН НАРЕЗНОЙ 300 Г</t>
+  </si>
+  <si>
+    <t>БАТОН НАРЕЗНОЙ (В НАРЕЗКЕ) 300 Г</t>
+  </si>
+  <si>
+    <t>БАТОН ОТРУБНОЙ 300 Г</t>
+  </si>
+  <si>
+    <t>БАТОН ОТРУБНОЙ (В НАРЕЗКЕ) 300 Г</t>
+  </si>
+  <si>
+    <t>БАТОН ТУРЕЦКИЙ 250 Г</t>
+  </si>
+  <si>
+    <t>БУЛОЧКА ДЛЯ ГАМБУРГЕРА 3 ШТ</t>
+  </si>
+  <si>
+    <t>БУЛОЧКА ДЛЯ ХОТ-ДОГА 3 ШТ</t>
+  </si>
+  <si>
+    <t>ГАЛЕТА, КГ</t>
+  </si>
+  <si>
+    <t>ЛАВАШ 2 ШТ</t>
+  </si>
+  <si>
+    <t>ЛЕПЕШКА РАМАЗАН 400 Г (Т)</t>
+  </si>
+  <si>
+    <t>ЛЕПЕШКА ТАШКЕНТСКАЯ 400 Г</t>
+  </si>
+  <si>
+    <t>СУХАРИ, КГ</t>
+  </si>
+  <si>
+    <t>ХЛЕБ БЕЗДРОЖЖЕВОЙ РЕМЕСЛЕННЫЙ 320 Г</t>
+  </si>
+  <si>
+    <t>ХЛЕБ КУКУРУЗНЫЙ (В НАРЕЗКЕ) 350 Г</t>
+  </si>
+  <si>
+    <t>ХЛЕБ КУКУРУЗНЫЙ 350 Г</t>
+  </si>
+  <si>
+    <t>ХЛЕБ ПОСОЛЬСКИЙ 400 Г</t>
+  </si>
+  <si>
+    <t>ХЛЕБ ПРЕЗИДЕНТСКИЙ (В НАРЕЗКЕ) 300 Г</t>
+  </si>
+  <si>
+    <t>ХЛЕБ ПРЕЗИДЕНТСКИЙ 300 Г</t>
+  </si>
+  <si>
+    <t>ХЛЕБ РЖАНОЙ НЕМЕЦКИЙ 400 Г</t>
+  </si>
+  <si>
+    <t>ХЛЕБ РОМАШКА С КУНЖУТОМ 300 Г</t>
+  </si>
+  <si>
+    <t>ХЛЕБ ТОСТОВЫЙ 300 Г</t>
+  </si>
+  <si>
+    <t>ХЛЕБ ЧЕСНОЧНЫЙ 200 Г</t>
+  </si>
+  <si>
+    <t>БУЛОЧКА СДОБНАЯ, КГ</t>
+  </si>
+  <si>
+    <t>БУЛОЧКИ С НАЧИНКОЙ, КГ</t>
+  </si>
+  <si>
+    <t>ХЛЕБЦЫ ЗЛАКОВЫЕ П/П, КГ</t>
+  </si>
+  <si>
+    <t>ПИРОЖКИ ЖАРЕНЫЕ С КАПУСТОЙ 80 Г</t>
+  </si>
+  <si>
+    <t>ПИРОЖКИ ЖАРЕНЫЕ С КАРТОШКОЙ 80 Г</t>
+  </si>
+  <si>
+    <t>ПИРОЖКИ ЖАРЕНЫЕ С ЛУКОМ/ЯЙЦОМ 100 Г</t>
+  </si>
+  <si>
+    <t>КАЛАЧ СМИТ ТУРЕЦКИЙ 1 ШТ</t>
+  </si>
+  <si>
+    <t>ПЛАЧИНДА С КУРИЦЕЙ 150Г</t>
+  </si>
+  <si>
+    <t>ПЛАЧИНДА С МЯСОМ 150Г</t>
+  </si>
+  <si>
+    <t>САМСА БОЛЬШАЯ С КУРИЦЕЙ 1 ШТ</t>
+  </si>
+  <si>
+    <t>САМСА БОЛЬШАЯ С МЯСОМ 1 ШТ</t>
+  </si>
+  <si>
+    <t>САМСА БОЛЬШАЯ С СЫРОМ 1 ШТ</t>
+  </si>
+  <si>
+    <t>САМСА УЙГУРСКАЯ С МЯСОМ 1 ШТ</t>
+  </si>
+  <si>
+    <t>САМСА МИКС 1 ШТ</t>
+  </si>
+  <si>
+    <t>САМСА ШАШЛЫК ФИЛЕ 1 ШТ</t>
+  </si>
+  <si>
+    <t>СЛОЙКА С СЫРОМ 140 Г</t>
+  </si>
+  <si>
+    <t>СЛОЙКА С ЯБЛОКОМ 140 Г</t>
+  </si>
+  <si>
+    <t>ТЕСТО ДЛЯ БАУРСАКОВ, КГ (1)</t>
+  </si>
+  <si>
+    <t>ТЕСТО СЛОЕНОЕ КЛАССИЧЕСКОЕ, КГ</t>
+  </si>
+  <si>
+    <t>БУЛОЧКА АЧМА С СЫРОМ 130 Г</t>
+  </si>
+  <si>
+    <t>БУЛОЧКА АЧМА С ШОКОЛАДОМ 130 Г</t>
+  </si>
+  <si>
+    <t>БУЛОЧКА АЧМА СО ШПИНАТОМ И ТВОРОГОМ 170 Г</t>
+  </si>
+  <si>
+    <t>БУЛОЧКА ПОАЧА С КАРТОШКОЙ 100 Г</t>
+  </si>
+  <si>
+    <t>БУЛОЧКА ПОАЧА С СЫРОМ 100 Г</t>
+  </si>
+  <si>
+    <t>БУЛОЧКА С ИЗЮМОМ 100Г</t>
+  </si>
+  <si>
+    <t>БУЛОЧКА С КОРИЦЕЙ 100Г</t>
+  </si>
+  <si>
+    <t>БУЛОЧКА ЯРОСЛАВСКАЯ 100 Г</t>
+  </si>
+  <si>
+    <t>БУЛОЧКА ВАТРУШКА 100Г</t>
+  </si>
+  <si>
+    <t>БУЛОЧКА СЕРДЕЧКО 100Г</t>
+  </si>
+  <si>
+    <t>БУЛОЧКА ПЛЕТЕНКА С МАКОМ 150 Г</t>
+  </si>
+  <si>
+    <t>ПЛЕТЕНКА СО СГУЩЕНКОЙ С ГРЕЦКИМ ОРЕХОМ 150 Г</t>
+  </si>
+  <si>
+    <t>ЭЛЕШ С КУРИЦЕЙ 150 Г</t>
+  </si>
+  <si>
+    <t>УЧПУЧМАК С МЯСОМ/КАРТОФЕЛЕМ 120 Г</t>
+  </si>
+  <si>
+    <t>СОСИСКА В ТЕСТЕ 100 Г</t>
+  </si>
+  <si>
+    <t>МИНИ ПИЦЦА НЕАПОЛИТАНСКАЯ ШТ 110 Г</t>
+  </si>
+  <si>
+    <t>МИНИ ПИЦЦА 130 Г (Т)</t>
+  </si>
+  <si>
+    <t>ЛЕПЕШКА С СЫРОМ 130 Г</t>
+  </si>
+  <si>
+    <t>СОСИСКА ПО-БАВАРСКИ 1 ШТ (В)</t>
+  </si>
+  <si>
+    <t>КРУАССАН С ШОКОЛАДОМ 100 Г</t>
+  </si>
+  <si>
+    <t>ПИРОЖКИ ПЕЧЕНЫЙ С КАПУСТОЙ 100 Г</t>
+  </si>
+  <si>
+    <t>ПИРОЖКИ ПЕЧЕНЫЙ С КАРТОШКОЙ 100 Г</t>
+  </si>
+  <si>
+    <t>ПИРОЖОК ПЕЧЕНЫЙ С ЯЙЦОМ ЛУКОМ 100 Г</t>
+  </si>
+  <si>
+    <t>ПИРОГ С КУРИЦЕЙ И КАРТОШКОЙ,КГ</t>
+  </si>
+  <si>
+    <t>ПИРОГ С МЯСОМ И КАРТОШКОЙ, КГ</t>
+  </si>
+  <si>
+    <t>БУЛОЧКА БЛИЗНЯШКА 150 Г</t>
   </si>
 </sst>
 </file>
@@ -1015,7 +1015,7 @@
         <v>99007445</v>
       </c>
       <c r="B1" t="s">
-        <v>55</v>
+        <v>134</v>
       </c>
       <c r="C1" s="5">
         <v>300</v>
@@ -1026,7 +1026,7 @@
         <v>99007481</v>
       </c>
       <c r="B2" t="s">
-        <v>107</v>
+        <v>135</v>
       </c>
       <c r="C2" s="5">
         <v>260</v>
@@ -1037,7 +1037,7 @@
         <v>99007482</v>
       </c>
       <c r="B3" t="s">
-        <v>108</v>
+        <v>136</v>
       </c>
       <c r="C3" s="5">
         <v>260</v>
@@ -1048,7 +1048,7 @@
         <v>99007508</v>
       </c>
       <c r="B4" t="s">
-        <v>120</v>
+        <v>137</v>
       </c>
       <c r="C4" s="5">
         <v>310</v>
@@ -1059,7 +1059,7 @@
         <v>99007509</v>
       </c>
       <c r="B5" t="s">
-        <v>121</v>
+        <v>138</v>
       </c>
       <c r="C5" s="5">
         <v>350</v>
@@ -1070,7 +1070,7 @@
         <v>99007510</v>
       </c>
       <c r="B6" t="s">
-        <v>122</v>
+        <v>139</v>
       </c>
       <c r="C6" s="5">
         <v>310</v>
@@ -1081,7 +1081,7 @@
         <v>99023828</v>
       </c>
       <c r="B7" t="s">
-        <v>124</v>
+        <v>140</v>
       </c>
       <c r="C7" s="5">
         <v>400</v>
@@ -1092,7 +1092,7 @@
         <v>99007511</v>
       </c>
       <c r="B8" t="s">
-        <v>123</v>
+        <v>141</v>
       </c>
       <c r="C8" s="5">
         <v>310</v>
@@ -1103,7 +1103,7 @@
         <v>99007513</v>
       </c>
       <c r="B9" t="s">
-        <v>125</v>
+        <v>142</v>
       </c>
       <c r="C9" s="5">
         <v>460</v>
@@ -1114,7 +1114,7 @@
         <v>99013240</v>
       </c>
       <c r="B10" t="s">
-        <v>126</v>
+        <v>143</v>
       </c>
       <c r="C10" s="5">
         <v>310</v>
@@ -1125,7 +1125,7 @@
         <v>99013263</v>
       </c>
       <c r="B11" t="s">
-        <v>127</v>
+        <v>144</v>
       </c>
       <c r="C11" s="5">
         <v>310</v>
@@ -1136,7 +1136,7 @@
         <v>99007488</v>
       </c>
       <c r="B12" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="C12" s="5">
         <v>850</v>
@@ -1147,7 +1147,7 @@
         <v>99007494</v>
       </c>
       <c r="B13" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="C13" s="5">
         <v>1000</v>
@@ -1158,7 +1158,7 @@
         <v>99013884</v>
       </c>
       <c r="B14" t="s">
-        <v>169</v>
+        <v>6</v>
       </c>
       <c r="C14" s="5">
         <v>600</v>
@@ -1169,7 +1169,7 @@
         <v>99013875</v>
       </c>
       <c r="B15" t="s">
-        <v>170</v>
+        <v>7</v>
       </c>
       <c r="C15" s="5">
         <v>600</v>
@@ -1180,7 +1180,7 @@
         <v>99007418</v>
       </c>
       <c r="B16" t="s">
-        <v>14</v>
+        <v>147</v>
       </c>
       <c r="C16" s="5">
         <v>350</v>
@@ -1191,7 +1191,7 @@
         <v>99014106</v>
       </c>
       <c r="B17" t="s">
-        <v>15</v>
+        <v>148</v>
       </c>
       <c r="C17" s="5">
         <v>350</v>
@@ -1202,7 +1202,7 @@
         <v>99014079</v>
       </c>
       <c r="B18" t="s">
-        <v>16</v>
+        <v>149</v>
       </c>
       <c r="C18" s="5">
         <v>500</v>
@@ -1213,7 +1213,7 @@
         <v>99020236</v>
       </c>
       <c r="B19" t="s">
-        <v>22</v>
+        <v>150</v>
       </c>
       <c r="C19" s="5">
         <v>240</v>
@@ -1224,7 +1224,7 @@
         <v>99020237</v>
       </c>
       <c r="B20" t="s">
-        <v>23</v>
+        <v>151</v>
       </c>
       <c r="C20" s="5">
         <v>300</v>
@@ -1235,7 +1235,7 @@
         <v>99007428</v>
       </c>
       <c r="B21" t="s">
-        <v>24</v>
+        <v>152</v>
       </c>
       <c r="C21" s="5">
         <v>220</v>
@@ -1246,7 +1246,7 @@
         <v>99007429</v>
       </c>
       <c r="B22" t="s">
-        <v>25</v>
+        <v>153</v>
       </c>
       <c r="C22" s="5">
         <v>220</v>
@@ -1257,7 +1257,7 @@
         <v>99007438</v>
       </c>
       <c r="B23" t="s">
-        <v>28</v>
+        <v>154</v>
       </c>
       <c r="C23" s="5">
         <v>220</v>
@@ -1268,7 +1268,7 @@
         <v>99007422</v>
       </c>
       <c r="B24" t="s">
-        <v>18</v>
+        <v>155</v>
       </c>
       <c r="C24" s="5">
         <v>200</v>
@@ -1279,7 +1279,7 @@
         <v>99007435</v>
       </c>
       <c r="B25" t="s">
-        <v>27</v>
+        <v>156</v>
       </c>
       <c r="C25" s="5">
         <v>220</v>
@@ -1290,7 +1290,7 @@
         <v>99007424</v>
       </c>
       <c r="B26" t="s">
-        <v>21</v>
+        <v>157</v>
       </c>
       <c r="C26" s="5">
         <v>300</v>
@@ -1301,7 +1301,7 @@
         <v>99029186</v>
       </c>
       <c r="B27" t="s">
-        <v>109</v>
+        <v>158</v>
       </c>
       <c r="C27" s="5">
         <v>260</v>
@@ -1312,7 +1312,7 @@
         <v>99024273</v>
       </c>
       <c r="B28" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="C28" s="5">
         <v>320</v>
@@ -1323,7 +1323,7 @@
         <v>99007495</v>
       </c>
       <c r="B29" t="s">
-        <v>141</v>
+        <v>160</v>
       </c>
       <c r="C29" s="5">
         <v>350</v>
@@ -1334,7 +1334,7 @@
         <v>99007484</v>
       </c>
       <c r="B30" t="s">
-        <v>128</v>
+        <v>161</v>
       </c>
       <c r="C30" s="5">
         <v>260</v>
@@ -1345,7 +1345,7 @@
         <v>99012643</v>
       </c>
       <c r="B31" t="s">
-        <v>74</v>
+        <v>162</v>
       </c>
       <c r="C31" s="5">
         <v>420</v>
@@ -1356,7 +1356,7 @@
         <v>99007468</v>
       </c>
       <c r="B32" t="s">
-        <v>73</v>
+        <v>163</v>
       </c>
       <c r="C32" s="5">
         <v>350</v>
@@ -1367,7 +1367,7 @@
         <v>99007461</v>
       </c>
       <c r="B33" t="s">
-        <v>69</v>
+        <v>164</v>
       </c>
       <c r="C33" s="5">
         <v>320</v>
@@ -1378,7 +1378,7 @@
         <v>99026674</v>
       </c>
       <c r="B34" t="s">
-        <v>129</v>
+        <v>165</v>
       </c>
       <c r="C34" s="5">
         <v>600</v>
@@ -1389,7 +1389,7 @@
         <v>99023606</v>
       </c>
       <c r="B35" t="s">
-        <v>62</v>
+        <v>166</v>
       </c>
       <c r="C35" s="5">
         <v>500</v>
@@ -1400,7 +1400,7 @@
         <v>99029431</v>
       </c>
       <c r="B36" t="s">
-        <v>104</v>
+        <v>167</v>
       </c>
       <c r="C36" s="5">
         <v>240</v>
@@ -1411,7 +1411,7 @@
         <v>99029430</v>
       </c>
       <c r="B37" t="s">
-        <v>105</v>
+        <v>168</v>
       </c>
       <c r="C37" s="5">
         <v>200</v>
@@ -1422,7 +1422,7 @@
         <v>99029429</v>
       </c>
       <c r="B38" t="s">
-        <v>106</v>
+        <v>169</v>
       </c>
       <c r="C38" s="5">
         <v>240</v>
@@ -1433,7 +1433,7 @@
         <v>99007472</v>
       </c>
       <c r="B39" t="s">
-        <v>97</v>
+        <v>170</v>
       </c>
       <c r="C39" s="5">
         <v>4000</v>
@@ -1444,7 +1444,7 @@
         <v>99007473</v>
       </c>
       <c r="B40" t="s">
-        <v>98</v>
+        <v>171</v>
       </c>
       <c r="C40" s="5">
         <v>4000</v>
@@ -1455,7 +1455,7 @@
         <v>99007421</v>
       </c>
       <c r="B41" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="C41" s="5">
         <v>390</v>
@@ -1481,7 +1481,7 @@
         <v>99022256</v>
       </c>
       <c r="B1" t="s">
-        <v>146</v>
+        <v>96</v>
       </c>
       <c r="C1">
         <v>500</v>
@@ -1492,7 +1492,7 @@
         <v>99014120</v>
       </c>
       <c r="B2" t="s">
-        <v>144</v>
+        <v>97</v>
       </c>
       <c r="C2">
         <v>400</v>
@@ -1503,7 +1503,7 @@
         <v>99029530</v>
       </c>
       <c r="B3" t="s">
-        <v>150</v>
+        <v>98</v>
       </c>
       <c r="C3">
         <v>600</v>
@@ -1514,7 +1514,7 @@
         <v>99007502</v>
       </c>
       <c r="B4" t="s">
-        <v>154</v>
+        <v>99</v>
       </c>
       <c r="C4">
         <v>260</v>
@@ -1525,7 +1525,7 @@
         <v>99020312</v>
       </c>
       <c r="B5" t="s">
-        <v>145</v>
+        <v>100</v>
       </c>
       <c r="C5">
         <v>220</v>
@@ -1536,7 +1536,7 @@
         <v>99013532</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>149</v>
+        <v>101</v>
       </c>
       <c r="C6">
         <v>210</v>
@@ -1547,7 +1547,7 @@
         <v>99007411</v>
       </c>
       <c r="B7" t="s">
-        <v>1</v>
+        <v>102</v>
       </c>
       <c r="C7">
         <v>300</v>
@@ -1558,7 +1558,7 @@
         <v>99022255</v>
       </c>
       <c r="B8" t="s">
-        <v>2</v>
+        <v>103</v>
       </c>
       <c r="C8">
         <v>380</v>
@@ -1569,7 +1569,7 @@
         <v>99007412</v>
       </c>
       <c r="B9" t="s">
-        <v>4</v>
+        <v>104</v>
       </c>
       <c r="C9">
         <v>240</v>
@@ -1580,7 +1580,7 @@
         <v>99028607</v>
       </c>
       <c r="B10" t="s">
-        <v>3</v>
+        <v>105</v>
       </c>
       <c r="C10">
         <v>250</v>
@@ -1591,7 +1591,7 @@
         <v>99007413</v>
       </c>
       <c r="B11" t="s">
-        <v>6</v>
+        <v>106</v>
       </c>
       <c r="C11">
         <v>220</v>
@@ -1602,7 +1602,7 @@
         <v>99028605</v>
       </c>
       <c r="B12" t="s">
-        <v>5</v>
+        <v>107</v>
       </c>
       <c r="C12">
         <v>240</v>
@@ -1613,7 +1613,7 @@
         <v>99007414</v>
       </c>
       <c r="B13" t="s">
-        <v>8</v>
+        <v>108</v>
       </c>
       <c r="C13">
         <v>220</v>
@@ -1624,7 +1624,7 @@
         <v>99028606</v>
       </c>
       <c r="B14" t="s">
-        <v>7</v>
+        <v>109</v>
       </c>
       <c r="C14">
         <v>240</v>
@@ -1635,7 +1635,7 @@
         <v>99007415</v>
       </c>
       <c r="B15" t="s">
-        <v>9</v>
+        <v>110</v>
       </c>
       <c r="C15">
         <v>200</v>
@@ -1646,7 +1646,7 @@
         <v>99022205</v>
       </c>
       <c r="B16" t="s">
-        <v>19</v>
+        <v>111</v>
       </c>
       <c r="C16">
         <v>270</v>
@@ -1657,7 +1657,7 @@
         <v>99022174</v>
       </c>
       <c r="B17" t="s">
-        <v>20</v>
+        <v>112</v>
       </c>
       <c r="C17">
         <v>270</v>
@@ -1668,7 +1668,7 @@
         <v>99022182</v>
       </c>
       <c r="B18" t="s">
-        <v>33</v>
+        <v>113</v>
       </c>
       <c r="C18">
         <v>1350</v>
@@ -1679,7 +1679,7 @@
         <v>99007459</v>
       </c>
       <c r="B19" t="s">
-        <v>64</v>
+        <v>114</v>
       </c>
       <c r="C19">
         <v>160</v>
@@ -1690,7 +1690,7 @@
         <v>99007460</v>
       </c>
       <c r="B20" t="s">
-        <v>68</v>
+        <v>115</v>
       </c>
       <c r="C20">
         <v>300</v>
@@ -1701,7 +1701,7 @@
         <v>99025638</v>
       </c>
       <c r="B21" t="s">
-        <v>70</v>
+        <v>116</v>
       </c>
       <c r="C21">
         <v>300</v>
@@ -1712,7 +1712,7 @@
         <v>99007486</v>
       </c>
       <c r="B22" t="s">
-        <v>132</v>
+        <v>117</v>
       </c>
       <c r="C22">
         <v>610</v>
@@ -1723,7 +1723,7 @@
         <v>99022254</v>
       </c>
       <c r="B23" t="s">
-        <v>143</v>
+        <v>118</v>
       </c>
       <c r="C23">
         <v>240</v>
@@ -1734,7 +1734,7 @@
         <v>99028609</v>
       </c>
       <c r="B24" t="s">
-        <v>147</v>
+        <v>119</v>
       </c>
       <c r="C24">
         <v>370</v>
@@ -1745,7 +1745,7 @@
         <v>99007501</v>
       </c>
       <c r="B25" t="s">
-        <v>148</v>
+        <v>120</v>
       </c>
       <c r="C25">
         <v>350</v>
@@ -1756,7 +1756,7 @@
         <v>99022478</v>
       </c>
       <c r="B26" t="s">
-        <v>151</v>
+        <v>121</v>
       </c>
       <c r="C26">
         <v>500</v>
@@ -1767,7 +1767,7 @@
         <v>99028610</v>
       </c>
       <c r="B27" t="s">
-        <v>152</v>
+        <v>122</v>
       </c>
       <c r="C27">
         <v>240</v>
@@ -1778,7 +1778,7 @@
         <v>99023189</v>
       </c>
       <c r="B28" t="s">
-        <v>153</v>
+        <v>123</v>
       </c>
       <c r="C28">
         <v>220</v>
@@ -1789,7 +1789,7 @@
         <v>99022257</v>
       </c>
       <c r="B29" t="s">
-        <v>155</v>
+        <v>124</v>
       </c>
       <c r="C29">
         <v>520</v>
@@ -1800,7 +1800,7 @@
         <v>99007503</v>
       </c>
       <c r="B30" t="s">
-        <v>156</v>
+        <v>125</v>
       </c>
       <c r="C30">
         <v>250</v>
@@ -1811,7 +1811,7 @@
         <v>99022294</v>
       </c>
       <c r="B31" t="s">
-        <v>157</v>
+        <v>126</v>
       </c>
       <c r="C31">
         <v>380</v>
@@ -1822,7 +1822,7 @@
         <v>99007505</v>
       </c>
       <c r="B32" t="s">
-        <v>158</v>
+        <v>127</v>
       </c>
       <c r="C32">
         <v>300</v>
@@ -1833,7 +1833,7 @@
         <v>99007434</v>
       </c>
       <c r="B33" t="s">
-        <v>26</v>
+        <v>128</v>
       </c>
       <c r="C33">
         <v>2000</v>
@@ -1844,7 +1844,7 @@
         <v>99007440</v>
       </c>
       <c r="B34" t="s">
-        <v>29</v>
+        <v>129</v>
       </c>
       <c r="C34">
         <v>2300</v>
@@ -1855,7 +1855,7 @@
         <v>99022252</v>
       </c>
       <c r="B35" t="s">
-        <v>159</v>
+        <v>130</v>
       </c>
       <c r="C35">
         <v>3500</v>
@@ -1866,7 +1866,7 @@
         <v>99024453</v>
       </c>
       <c r="B36" t="s">
-        <v>101</v>
+        <v>131</v>
       </c>
       <c r="C36">
         <v>200</v>
@@ -1877,7 +1877,7 @@
         <v>99024452</v>
       </c>
       <c r="B37" t="s">
-        <v>102</v>
+        <v>132</v>
       </c>
       <c r="C37">
         <v>200</v>
@@ -1888,7 +1888,7 @@
         <v>99024455</v>
       </c>
       <c r="B38" t="s">
-        <v>103</v>
+        <v>133</v>
       </c>
       <c r="C38">
         <v>200</v>
@@ -1913,7 +1913,7 @@
         <v>99014010</v>
       </c>
       <c r="B1" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C1" s="5">
         <v>200</v>
@@ -1924,7 +1924,7 @@
         <v>99026922</v>
       </c>
       <c r="B2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C2" s="5">
         <v>220</v>
@@ -1935,7 +1935,7 @@
         <v>99019055</v>
       </c>
       <c r="B3" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="C3" s="5">
         <v>1000</v>
@@ -1946,7 +1946,7 @@
         <v>99024662</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C4" s="6">
         <v>500</v>
@@ -1957,7 +1957,7 @@
         <v>99025975</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C5" s="6">
         <v>500</v>
@@ -1968,7 +1968,7 @@
         <v>99002867</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C6" s="6">
         <v>500</v>
@@ -1979,7 +1979,7 @@
         <v>99009484</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C7" s="6">
         <v>500</v>
@@ -1990,7 +1990,7 @@
         <v>99008289</v>
       </c>
       <c r="B8" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C8" s="5">
         <v>846</v>
@@ -2001,7 +2001,7 @@
         <v>99008248</v>
       </c>
       <c r="B9" t="s">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="C9" s="5">
         <v>600</v>
@@ -2012,7 +2012,7 @@
         <v>99008673</v>
       </c>
       <c r="B10" t="s">
-        <v>54</v>
+        <v>77</v>
       </c>
       <c r="C10" s="5">
         <v>600</v>
@@ -2023,7 +2023,7 @@
         <v>99009926</v>
       </c>
       <c r="B11" t="s">
-        <v>0</v>
+        <v>78</v>
       </c>
       <c r="C11" s="5">
         <v>710</v>
@@ -2034,7 +2034,7 @@
         <v>99011503</v>
       </c>
       <c r="B12" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="C12" s="5">
         <v>1200</v>
@@ -2045,7 +2045,7 @@
         <v>99011505</v>
       </c>
       <c r="B13" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="C13" s="5">
         <v>1400</v>
@@ -2056,7 +2056,7 @@
         <v>99025834</v>
       </c>
       <c r="B14" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C14" s="5">
         <v>3300</v>
@@ -2067,7 +2067,7 @@
         <v>99025591</v>
       </c>
       <c r="B15" t="s">
-        <v>131</v>
+        <v>82</v>
       </c>
       <c r="C15" s="5">
         <v>14500</v>
@@ -2078,7 +2078,7 @@
         <v>99007347</v>
       </c>
       <c r="B16" t="s">
-        <v>13</v>
+        <v>83</v>
       </c>
       <c r="C16" s="5">
         <v>2000</v>
@@ -2089,7 +2089,7 @@
         <v>99025572</v>
       </c>
       <c r="B17" t="s">
-        <v>111</v>
+        <v>84</v>
       </c>
       <c r="C17" s="5">
         <v>3600</v>
@@ -2100,7 +2100,7 @@
         <v>99025573</v>
       </c>
       <c r="B18" t="s">
-        <v>66</v>
+        <v>85</v>
       </c>
       <c r="C18" s="5">
         <v>3600</v>
@@ -2111,7 +2111,7 @@
         <v>99022395</v>
       </c>
       <c r="B19" t="s">
-        <v>10</v>
+        <v>86</v>
       </c>
       <c r="C19" s="5">
         <v>1200</v>
@@ -2122,7 +2122,7 @@
         <v>99020261</v>
       </c>
       <c r="B20" t="s">
-        <v>56</v>
+        <v>87</v>
       </c>
       <c r="C20" s="5">
         <v>1700</v>
@@ -2133,7 +2133,7 @@
         <v>99022365</v>
       </c>
       <c r="B21" t="s">
-        <v>67</v>
+        <v>88</v>
       </c>
       <c r="C21" s="5">
         <v>2300</v>
@@ -2144,7 +2144,7 @@
         <v>99023040</v>
       </c>
       <c r="B22" t="s">
-        <v>171</v>
+        <v>8</v>
       </c>
       <c r="C22" s="5">
         <v>2500</v>
@@ -2155,7 +2155,7 @@
         <v>99027074</v>
       </c>
       <c r="B23" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="C23" s="5">
         <v>2300</v>
@@ -2166,7 +2166,7 @@
         <v>99013997</v>
       </c>
       <c r="B24" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C24" s="7">
         <v>3200</v>
@@ -2177,7 +2177,7 @@
         <v>99011506</v>
       </c>
       <c r="B25" t="s">
-        <v>133</v>
+        <v>91</v>
       </c>
       <c r="C25" s="5">
         <v>300</v>
@@ -2188,7 +2188,7 @@
         <v>99013864</v>
       </c>
       <c r="B26" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="C26" s="5">
         <v>1840</v>
@@ -2199,7 +2199,7 @@
         <v>99008004</v>
       </c>
       <c r="B27" t="s">
-        <v>57</v>
+        <v>93</v>
       </c>
       <c r="C27" s="5">
         <v>3500</v>
@@ -2210,7 +2210,7 @@
         <v>99025569</v>
       </c>
       <c r="B28" t="s">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="C28" s="5">
         <v>3600</v>
@@ -2221,7 +2221,7 @@
         <v>99009553</v>
       </c>
       <c r="B29" t="s">
-        <v>63</v>
+        <v>95</v>
       </c>
       <c r="C29" s="5">
         <v>390</v>
@@ -2249,7 +2249,7 @@
         <v>2175106</v>
       </c>
       <c r="B1" t="s">
-        <v>163</v>
+        <v>0</v>
       </c>
       <c r="C1" s="5">
         <v>3000</v>
@@ -2260,7 +2260,7 @@
         <v>2134467</v>
       </c>
       <c r="B2" t="s">
-        <v>164</v>
+        <v>1</v>
       </c>
       <c r="C2" s="5">
         <v>3600</v>
@@ -2271,7 +2271,7 @@
         <v>2126236</v>
       </c>
       <c r="B3" t="s">
-        <v>165</v>
+        <v>2</v>
       </c>
       <c r="C3" s="5">
         <v>3000</v>
@@ -2282,7 +2282,7 @@
         <v>2109176</v>
       </c>
       <c r="B4" t="s">
-        <v>166</v>
+        <v>3</v>
       </c>
       <c r="C4" s="5">
         <v>2200</v>
@@ -2293,7 +2293,7 @@
         <v>2120835</v>
       </c>
       <c r="B5" t="s">
-        <v>167</v>
+        <v>4</v>
       </c>
       <c r="C5" s="5">
         <v>4000</v>
@@ -2304,7 +2304,7 @@
         <v>9001003004</v>
       </c>
       <c r="B6" t="s">
-        <v>168</v>
+        <v>5</v>
       </c>
       <c r="C6" s="5">
         <v>4000</v>
@@ -2315,7 +2315,7 @@
         <v>99024274</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>172</v>
+        <v>9</v>
       </c>
       <c r="C7" s="6">
         <v>2500</v>
@@ -2326,7 +2326,7 @@
         <v>99023895</v>
       </c>
       <c r="B8" t="s">
-        <v>119</v>
+        <v>67</v>
       </c>
       <c r="C8" s="5">
         <v>1500</v>
@@ -2351,7 +2351,7 @@
         <v>99008243</v>
       </c>
       <c r="B1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C1" s="5">
         <v>1300</v>
@@ -2362,7 +2362,7 @@
         <v>99008176</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C2" s="5">
         <v>1300</v>
@@ -2373,7 +2373,7 @@
         <v>99003502</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="C3" s="5">
         <v>3750</v>
@@ -2384,7 +2384,7 @@
         <v>99023335</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="C4" s="5">
         <v>4000</v>
@@ -2395,7 +2395,7 @@
         <v>99003503</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C5" s="5">
         <v>3300</v>
@@ -2406,7 +2406,7 @@
         <v>99007449</v>
       </c>
       <c r="B6" t="s">
-        <v>58</v>
+        <v>34</v>
       </c>
       <c r="C6" s="5">
         <v>450</v>
@@ -2417,7 +2417,7 @@
         <v>99007449</v>
       </c>
       <c r="B7" t="s">
-        <v>58</v>
+        <v>34</v>
       </c>
       <c r="C7" s="5">
         <v>450</v>
@@ -2428,7 +2428,7 @@
         <v>99007457</v>
       </c>
       <c r="B8" t="s">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="C8" s="5">
         <v>400</v>
@@ -2439,7 +2439,7 @@
         <v>99013089</v>
       </c>
       <c r="B9" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="C9" s="5">
         <v>600</v>
@@ -2450,7 +2450,7 @@
         <v>99023014</v>
       </c>
       <c r="B10" t="s">
-        <v>59</v>
+        <v>37</v>
       </c>
       <c r="C10" s="5">
         <v>3000</v>
@@ -2461,7 +2461,7 @@
         <v>99023015</v>
       </c>
       <c r="B11" t="s">
-        <v>161</v>
+        <v>38</v>
       </c>
       <c r="C11" s="5">
         <v>250</v>
@@ -2472,7 +2472,7 @@
         <v>99022604</v>
       </c>
       <c r="B12" t="s">
-        <v>113</v>
+        <v>39</v>
       </c>
       <c r="C12" s="5">
         <v>3600</v>
@@ -2483,7 +2483,7 @@
         <v>99028639</v>
       </c>
       <c r="B13" t="s">
-        <v>96</v>
+        <v>40</v>
       </c>
       <c r="C13" s="5">
         <v>3700</v>
@@ -2494,7 +2494,7 @@
         <v>99022876</v>
       </c>
       <c r="B14" t="s">
-        <v>99</v>
+        <v>41</v>
       </c>
       <c r="C14" s="5">
         <v>3700</v>
@@ -2505,7 +2505,7 @@
         <v>99007475</v>
       </c>
       <c r="B15" t="s">
-        <v>100</v>
+        <v>42</v>
       </c>
       <c r="C15" s="5">
         <v>3000</v>
@@ -2516,7 +2516,7 @@
         <v>99026664</v>
       </c>
       <c r="B16" t="s">
-        <v>118</v>
+        <v>43</v>
       </c>
       <c r="C16" s="5">
         <v>610</v>
@@ -2527,7 +2527,7 @@
         <v>99025467</v>
       </c>
       <c r="B17" t="s">
-        <v>114</v>
+        <v>44</v>
       </c>
       <c r="C17" s="5">
         <v>510</v>
@@ -2538,7 +2538,7 @@
         <v>99025468</v>
       </c>
       <c r="B18" t="s">
-        <v>117</v>
+        <v>45</v>
       </c>
       <c r="C18" s="5">
         <v>550</v>
@@ -2549,7 +2549,7 @@
         <v>99023084</v>
       </c>
       <c r="B19" t="s">
-        <v>115</v>
+        <v>46</v>
       </c>
       <c r="C19" s="5">
         <v>3000</v>
@@ -2560,7 +2560,7 @@
         <v>99023190</v>
       </c>
       <c r="B20" t="s">
-        <v>116</v>
+        <v>47</v>
       </c>
       <c r="C20" s="5">
         <v>3000</v>
@@ -2571,7 +2571,7 @@
         <v>99007485</v>
       </c>
       <c r="B21" t="s">
-        <v>130</v>
+        <v>48</v>
       </c>
       <c r="C21" s="5">
         <v>300</v>
@@ -2582,7 +2582,7 @@
         <v>99029423</v>
       </c>
       <c r="B22" t="s">
-        <v>140</v>
+        <v>49</v>
       </c>
       <c r="C22" s="5">
         <v>1000</v>
@@ -2593,7 +2593,7 @@
         <v>99023773</v>
       </c>
       <c r="B23" t="s">
-        <v>142</v>
+        <v>50</v>
       </c>
       <c r="C23" s="5">
         <v>3000</v>
@@ -2604,7 +2604,7 @@
         <v>99003519</v>
       </c>
       <c r="B24" t="s">
-        <v>160</v>
+        <v>51</v>
       </c>
       <c r="C24" s="5">
         <v>3000</v>
@@ -2615,7 +2615,7 @@
         <v>99008144</v>
       </c>
       <c r="B25" t="s">
-        <v>112</v>
+        <v>52</v>
       </c>
       <c r="C25" s="5">
         <v>320</v>
@@ -2626,7 +2626,7 @@
         <v>99008201</v>
       </c>
       <c r="B26" t="s">
-        <v>136</v>
+        <v>53</v>
       </c>
       <c r="C26" s="5">
         <v>2580</v>
@@ -2637,7 +2637,7 @@
         <v>99026270</v>
       </c>
       <c r="B27" t="s">
-        <v>137</v>
+        <v>54</v>
       </c>
       <c r="C27" s="5">
         <v>2500</v>
@@ -2648,7 +2648,7 @@
         <v>99029164</v>
       </c>
       <c r="B28" t="s">
-        <v>138</v>
+        <v>55</v>
       </c>
       <c r="C28" s="5">
         <v>3600</v>
@@ -2659,7 +2659,7 @@
         <v>99011851</v>
       </c>
       <c r="B29" t="s">
-        <v>139</v>
+        <v>56</v>
       </c>
       <c r="C29" s="5">
         <v>3600</v>
@@ -2670,7 +2670,7 @@
         <v>99025611</v>
       </c>
       <c r="B30" t="s">
-        <v>86</v>
+        <v>57</v>
       </c>
       <c r="C30" s="5">
         <v>3000</v>
@@ -2681,7 +2681,7 @@
         <v>99003505</v>
       </c>
       <c r="B31" t="s">
-        <v>91</v>
+        <v>58</v>
       </c>
       <c r="C31" s="5">
         <v>3200</v>
@@ -2692,7 +2692,7 @@
         <v>99013871</v>
       </c>
       <c r="B32" t="s">
-        <v>90</v>
+        <v>59</v>
       </c>
       <c r="C32" s="5">
         <v>4000</v>
@@ -2703,7 +2703,7 @@
         <v>99025612</v>
       </c>
       <c r="B33" t="s">
-        <v>89</v>
+        <v>60</v>
       </c>
       <c r="C33" s="5">
         <v>2100</v>
@@ -2714,7 +2714,7 @@
         <v>99003507</v>
       </c>
       <c r="B34" t="s">
-        <v>92</v>
+        <v>61</v>
       </c>
       <c r="C34" s="5">
         <v>3000</v>
@@ -2725,7 +2725,7 @@
         <v>99025609</v>
       </c>
       <c r="B35" t="s">
-        <v>93</v>
+        <v>62</v>
       </c>
       <c r="C35" s="5">
         <v>2500</v>
@@ -2736,7 +2736,7 @@
         <v>99003504</v>
       </c>
       <c r="B36" t="s">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="C36" s="5">
         <v>2400</v>
@@ -2747,7 +2747,7 @@
         <v>99003513</v>
       </c>
       <c r="B37" t="s">
-        <v>94</v>
+        <v>64</v>
       </c>
       <c r="C37" s="5">
         <v>2400</v>
@@ -2758,7 +2758,7 @@
         <v>99003514</v>
       </c>
       <c r="B38" t="s">
-        <v>95</v>
+        <v>65</v>
       </c>
       <c r="C38" s="5">
         <v>2400</v>
@@ -2769,7 +2769,7 @@
         <v>99023336</v>
       </c>
       <c r="B39" t="s">
-        <v>87</v>
+        <v>66</v>
       </c>
       <c r="C39" s="5">
         <v>2400</v>
@@ -2794,7 +2794,7 @@
         <v>99027720</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="C1" s="7">
         <v>1150</v>
@@ -2805,7 +2805,7 @@
         <v>99008102</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="C2" s="7">
         <v>1150</v>
@@ -2816,7 +2816,7 @@
         <v>99027357</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="C3" s="7">
         <v>1150</v>
@@ -2827,7 +2827,7 @@
         <v>99027719</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="C4" s="7">
         <v>1150</v>
@@ -2838,7 +2838,7 @@
         <v>99027721</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="C5" s="7">
         <v>1150</v>
@@ -2849,7 +2849,7 @@
         <v>99027722</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="C6" s="7">
         <v>1150</v>
@@ -2860,7 +2860,7 @@
         <v>99008094</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="C7" s="7">
         <v>1150</v>
@@ -2871,7 +2871,7 @@
         <v>99027354</v>
       </c>
       <c r="B8" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="C8" s="7">
         <v>1150</v>
@@ -2882,7 +2882,7 @@
         <v>99027353</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>18</v>
       </c>
       <c r="C9" s="7">
         <v>1150</v>
@@ -2893,7 +2893,7 @@
         <v>99007712</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="C10" s="7">
         <v>1150</v>
@@ -2904,7 +2904,7 @@
         <v>99008096</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="C11" s="7">
         <v>1150</v>
@@ -2915,7 +2915,7 @@
         <v>99008099</v>
       </c>
       <c r="B12" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="C12" s="7">
         <v>1150</v>
@@ -2926,7 +2926,7 @@
         <v>99007713</v>
       </c>
       <c r="B13" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="C13" s="7">
         <v>1150</v>
@@ -2937,7 +2937,7 @@
         <v>99007725</v>
       </c>
       <c r="B14" t="s">
-        <v>47</v>
+        <v>23</v>
       </c>
       <c r="C14" s="7">
         <v>1150</v>
@@ -2948,7 +2948,7 @@
         <v>99027355</v>
       </c>
       <c r="B15" t="s">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="C15" s="7">
         <v>1150</v>
@@ -2959,7 +2959,7 @@
         <v>99028729</v>
       </c>
       <c r="B16" t="s">
-        <v>49</v>
+        <v>25</v>
       </c>
       <c r="C16" s="7">
         <v>1150</v>
@@ -2970,7 +2970,7 @@
         <v>99028987</v>
       </c>
       <c r="B17" t="s">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="C17" s="7">
         <v>1200</v>
@@ -2981,7 +2981,7 @@
         <v>99027723</v>
       </c>
       <c r="B18" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="C18" s="7">
         <v>1150</v>
@@ -2992,7 +2992,7 @@
         <v>99007728</v>
       </c>
       <c r="B19" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="C19" s="7">
         <v>1150</v>

</xml_diff>